<commit_message>
chore: add dockerignore configuration, error analysis script, and template files
</commit_message>
<xml_diff>
--- a/test_template.xlsx
+++ b/test_template.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cabecalho" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Itens" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cabecalho" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Itens" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,7 +29,19 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="3">
@@ -57,11 +70,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -136,6 +152,96 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Sistema</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Número da nota fiscal de entrada que será gerada. Ex: 12345</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Data de emissão da nota.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Data de entrada das mercadorias.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>CFOP principal da nota (Ex: 3101). Irá no cabeçalho.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Número do Pedido de Compra (Campo 44 do Layout).</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Percentual de redução da base de ICMS (Campo 45).</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Código do Importador no sistema destino.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Código do Transportador no sistema destino.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Código do Exportador no sistema destino.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Sistema</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>O código NCM de 8 dígitos presente no XML. Este é o campo chave para o mapeamento.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Descrição do produto. Este campo é apenas para referência e não é usado pelo sistema.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>O código do produto no seu sistema ERP. (Obrigatório)</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Unidade de medida que deve constar na nota (ex: UN, CX, KG). Se vazio, usará a unidade do XML.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>CFOP de entrada da mercadoria. (Obrigatório)</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -427,50 +533,168 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Numero da Nota (Obrigatorio)</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Data Emissao (DD/MM/AAAA)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Data Entrada (DD/MM/AAAA)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Valor Frete Total (Opcional)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Valor Seguro Total (Opcional)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Nome Exportador (Opcional)</t>
+          <t>Guia de Preenchimento do Modelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo do Modelo:</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Este modelo serve para complementar os dados da Declaração de Importação (DI) XML com informações internas do seu sistema (códigos de produto, CFOPs) e para definir dados da nota fiscal que não existem no XML.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Guia Rápido:</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1. Preencha a aba 'Cabecalho' com os dados da sua nota fiscal (Número e Datas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2. Na aba 'Itens', mapeie cada NCM do seu XML para o código de produto interno e CFOP correspondente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>3. Salve o arquivo e faça o upload na aplicação junto com o XML da DI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>4. Importante: A ordem das colunas deve ser mantida. Não adicione, remova ou reordene.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>5. A ordem das linhas na aba 'Itens' não importa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Histórico de Versões:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Versão</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Alteração</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>22/01/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Versão inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>23/01/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Adicionado guia de preenchimento e exemplos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>23/01/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Adicionada nota sobre a ordem das colunas e linhas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>23/01/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Simplificado template. Frete, Seguro e Exportador agora são lidos do XML.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -481,7 +705,127 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Numero da Nota (Obrigatorio)</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Data Emissao (DD/MM/AAAA)</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Data Entrada (DD/MM/AAAA)</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>CFOP Predominante (Obrigatorio)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Numero do PO (Opcional)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Perc Reducao ICMS (Opcional)</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Codigo Importador (Opcional)</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Codigo Transportador (Opcional)</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Codigo Exportador (Opcional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>23/01/2026</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>24/01/2026</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>3101</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>PO-999</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>IMP-001</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>TRA-002</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>EXP-003</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -492,33 +836,61 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Codigo NCM (XML)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Descricao (XML - Opcional)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Codigo Produto Interno (Obrigatorio)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Unidade Saida (Opcional)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>CFOP (Obrigatorio)</t>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Descricao (Informativo)</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Codigo Produto Interno</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Unidade Saida</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>CFOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>85171231</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Smartphone Modelo X</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>PROD-00123</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>3101</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>